<commit_message>
fix: ofertowanie_export — Grupa kartoteki wyklucza galaz 10_Oferty (OfferingTree CTE)
</commit_message>
<xml_diff>
--- a/output/ofertowanie_2025_/_AUCHAN_2026-03-30.xlsx
+++ b/output/ofertowanie_2025_/_AUCHAN_2026-03-30.xlsx
@@ -1138,7 +1138,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1692,7 +1692,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -2388,7 +2388,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -2802,7 +2802,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -3009,7 +3009,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -3275,7 +3275,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>AUCHAN</t>
+          <t>\10_OFERTY\2025\AUCHAN</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix: ofertowanie_export — Grupa kartoteki filtr LIKE Cmentarz (pelna sciezka)
</commit_message>
<xml_diff>
--- a/output/ofertowanie_2025_/_AUCHAN_2026-03-30.xlsx
+++ b/output/ofertowanie_2025_/_AUCHAN_2026-03-30.xlsx
@@ -1138,7 +1138,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1692,7 +1692,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -2388,7 +2388,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -2802,7 +2802,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -3009,7 +3009,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -3275,7 +3275,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>\10_OFERTY\2025\AUCHAN</t>
+          <t>\Cmentarz\Znicze\Solarne</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">

</xml_diff>